<commit_message>
cn-#14 proper handling after table line which has contents at the tailing columns.
</commit_message>
<xml_diff>
--- a/test/Cactus.ReqnrollConveterTest/Features/DataGridSample.xlsx
+++ b/test/Cactus.ReqnrollConveterTest/Features/DataGridSample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\itu\Cactus.net\test\Cactus.ReqnrollConveterTest\Features\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7710C3F8-B2AE-4403-9B31-E194C58FB220}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EB04D0F-8F14-4265-9F76-4BE7CCC6FF99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-2985" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AddTwoNumbers" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="SumProduct" sheetId="2" r:id="rId3"/>
     <sheet name="SumAverage" sheetId="3" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029" iterateCount="250" iterateDelta="1.0000000000000001E-5"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="26">
   <si>
     <t>Scenario</t>
   </si>
@@ -634,6 +634,11 @@
         <v>12</v>
       </c>
     </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+    </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>

</xml_diff>